<commit_message>
refactor: update excel export templates and debugging
Updated RFS and PIS excel templates and added diagnostic logging to the template export utility to facilitate troubleshooting of formula and cell value rendering.
</commit_message>
<xml_diff>
--- a/public/templates/PIS_TEMPLATE.xlsx
+++ b/public/templates/PIS_TEMPLATE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/59650d1564ea21d1/Desktop/System Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{62ED0C2D-6914-47B8-814B-71FF416C8C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02AA02E7-B82A-4785-B500-24D11D28E9A8}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{62ED0C2D-6914-47B8-814B-71FF416C8C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11C82A08-96BB-4F1D-92CA-E03C4AA5C589}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,14 +34,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
   <si>
     <t>SMEI Payment Instruction Slip</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
     <t>AM</t>
   </si>
   <si>
@@ -55,9 +52,6 @@
   </si>
   <si>
     <t>Amount</t>
-  </si>
-  <si>
-    <t>x</t>
   </si>
   <si>
     <t>Php</t>
@@ -626,6 +620,9 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -640,69 +637,66 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="15" fontId="4" fillId="0" borderId="3" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="15" fontId="4" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1013,31 +1007,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="28.2" thickBot="1">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="53"/>
-      <c r="G1" s="53"/>
-      <c r="H1" s="53"/>
-      <c r="I1" s="53"/>
-      <c r="J1" s="53"/>
-      <c r="K1" s="53"/>
-      <c r="L1" s="53"/>
-      <c r="M1" s="53"/>
-      <c r="N1" s="54" t="s">
-        <v>28</v>
-      </c>
-      <c r="O1" s="54"/>
-      <c r="P1" s="54"/>
-      <c r="Q1" s="54"/>
-      <c r="R1" s="54"/>
-      <c r="S1" s="54"/>
-      <c r="T1" s="54"/>
-      <c r="U1" s="55"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
+      <c r="K1" s="54"/>
+      <c r="L1" s="54"/>
+      <c r="M1" s="54"/>
+      <c r="N1" s="55" t="s">
+        <v>26</v>
+      </c>
+      <c r="O1" s="55"/>
+      <c r="P1" s="55"/>
+      <c r="Q1" s="55"/>
+      <c r="R1" s="55"/>
+      <c r="S1" s="55"/>
+      <c r="T1" s="55"/>
+      <c r="U1" s="56"/>
     </row>
     <row r="2" spans="1:21" ht="3.75" customHeight="1"/>
     <row r="3" spans="1:21">
@@ -1054,37 +1048,35 @@
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
-      <c r="N3" s="3" t="s">
-        <v>1</v>
-      </c>
+      <c r="N3" s="3"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q3" s="2"/>
       <c r="R3" s="2"/>
       <c r="S3" s="26"/>
       <c r="T3" s="2"/>
       <c r="U3" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="17.399999999999999">
       <c r="A4" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
-      <c r="F4" s="72" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="56"/>
-      <c r="H4" s="56"/>
-      <c r="I4" s="56"/>
-      <c r="J4" s="56"/>
-      <c r="K4" s="56"/>
+      <c r="F4" s="57" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
+      <c r="J4" s="58"/>
+      <c r="K4" s="58"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
@@ -1098,13 +1090,13 @@
     </row>
     <row r="5" spans="1:21" ht="17.399999999999999">
       <c r="A5" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="47"/>
       <c r="C5" s="48"/>
       <c r="D5" s="48"/>
       <c r="E5" s="48" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F5" s="48"/>
       <c r="G5" s="48"/>
@@ -1148,40 +1140,38 @@
     </row>
     <row r="7" spans="1:21" ht="16.2">
       <c r="A7" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="2"/>
-      <c r="C7" s="3" t="s">
-        <v>7</v>
-      </c>
+      <c r="C7" s="3"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I7" s="24"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L7" s="24"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
-      <c r="Q7" s="57">
+      <c r="Q7" s="59">
         <v>0</v>
       </c>
-      <c r="R7" s="57"/>
-      <c r="S7" s="57"/>
-      <c r="T7" s="57"/>
-      <c r="U7" s="57"/>
+      <c r="R7" s="59"/>
+      <c r="S7" s="59"/>
+      <c r="T7" s="59"/>
+      <c r="U7" s="59"/>
     </row>
     <row r="8" spans="1:21">
       <c r="A8" s="2"/>
@@ -1208,13 +1198,13 @@
     </row>
     <row r="9" spans="1:21">
       <c r="A9" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="3"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -1222,7 +1212,7 @@
       <c r="I9" s="3"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
@@ -1232,7 +1222,7 @@
       <c r="Q9" s="50"/>
       <c r="R9" s="2"/>
       <c r="S9" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="T9" s="2"/>
       <c r="U9" s="2"/>
@@ -1266,7 +1256,7 @@
       <c r="C11" s="3"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -1274,18 +1264,18 @@
       <c r="I11" s="3"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
-      <c r="Q11" s="58"/>
-      <c r="R11" s="58"/>
-      <c r="S11" s="58"/>
-      <c r="T11" s="58"/>
-      <c r="U11" s="58"/>
+      <c r="Q11" s="60"/>
+      <c r="R11" s="60"/>
+      <c r="S11" s="60"/>
+      <c r="T11" s="60"/>
+      <c r="U11" s="60"/>
     </row>
     <row r="12" spans="1:21">
       <c r="A12" s="2"/>
@@ -1312,10 +1302,10 @@
     </row>
     <row r="13" spans="1:21">
       <c r="A13" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -1348,13 +1338,13 @@
       <c r="H14" s="43"/>
       <c r="I14" s="43"/>
       <c r="J14" s="45"/>
-      <c r="K14" s="73" t="s">
-        <v>34</v>
+      <c r="K14" s="51" t="s">
+        <v>32</v>
       </c>
       <c r="L14" s="43"/>
       <c r="M14" s="43"/>
       <c r="N14" s="43" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="O14" s="43"/>
       <c r="P14" s="43"/>
@@ -1363,7 +1353,7 @@
       <c r="S14" s="43"/>
       <c r="T14" s="43"/>
       <c r="U14" s="43" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:21">
@@ -1378,22 +1368,22 @@
       <c r="I15" s="10"/>
       <c r="J15" s="7"/>
       <c r="K15" s="46" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="L15" s="7"/>
       <c r="M15" s="30"/>
-      <c r="N15" s="75" t="s">
-        <v>38</v>
-      </c>
-      <c r="O15" s="74"/>
-      <c r="P15" s="74"/>
-      <c r="Q15" s="74"/>
-      <c r="R15" s="74"/>
-      <c r="S15" s="74"/>
-      <c r="T15" s="10"/>
-      <c r="U15" s="76" t="s">
-        <v>39</v>
-      </c>
+      <c r="N15" s="61" t="s">
+        <v>36</v>
+      </c>
+      <c r="O15" s="62"/>
+      <c r="P15" s="62"/>
+      <c r="Q15" s="62"/>
+      <c r="R15" s="62"/>
+      <c r="S15" s="62"/>
+      <c r="T15" s="76" t="s">
+        <v>37</v>
+      </c>
+      <c r="U15" s="76"/>
     </row>
     <row r="16" spans="1:21">
       <c r="A16" s="31"/>
@@ -1409,12 +1399,12 @@
       <c r="K16" s="40"/>
       <c r="L16" s="31"/>
       <c r="M16" s="33"/>
-      <c r="N16" s="59"/>
-      <c r="O16" s="59"/>
-      <c r="P16" s="59"/>
-      <c r="Q16" s="59"/>
-      <c r="R16" s="59"/>
-      <c r="S16" s="59"/>
+      <c r="N16" s="65"/>
+      <c r="O16" s="65"/>
+      <c r="P16" s="65"/>
+      <c r="Q16" s="65"/>
+      <c r="R16" s="65"/>
+      <c r="S16" s="65"/>
       <c r="T16" s="31"/>
       <c r="U16" s="31"/>
     </row>
@@ -1432,12 +1422,12 @@
       <c r="K17" s="39"/>
       <c r="L17" s="6"/>
       <c r="M17" s="29"/>
-      <c r="N17" s="62"/>
-      <c r="O17" s="62"/>
-      <c r="P17" s="62"/>
-      <c r="Q17" s="62"/>
-      <c r="R17" s="62"/>
-      <c r="S17" s="62"/>
+      <c r="N17" s="66"/>
+      <c r="O17" s="66"/>
+      <c r="P17" s="66"/>
+      <c r="Q17" s="66"/>
+      <c r="R17" s="66"/>
+      <c r="S17" s="66"/>
       <c r="T17" s="6"/>
       <c r="U17" s="6"/>
     </row>
@@ -1449,8 +1439,8 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
-      <c r="H18" s="63"/>
-      <c r="I18" s="63"/>
+      <c r="H18" s="67"/>
+      <c r="I18" s="67"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -1466,7 +1456,7 @@
     </row>
     <row r="19" spans="1:21">
       <c r="A19" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1479,7 +1469,7 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
@@ -1511,64 +1501,64 @@
       <c r="Q20" s="2"/>
       <c r="R20" s="2"/>
       <c r="S20" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
     </row>
     <row r="21" spans="1:21">
-      <c r="A21" s="60" t="s">
-        <v>32</v>
-      </c>
-      <c r="B21" s="60"/>
-      <c r="C21" s="60"/>
-      <c r="D21" s="60"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="60"/>
-      <c r="H21" s="60"/>
+      <c r="A21" s="63" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="63"/>
+      <c r="C21" s="63"/>
+      <c r="D21" s="63"/>
+      <c r="E21" s="63"/>
+      <c r="F21" s="63"/>
+      <c r="G21" s="63"/>
+      <c r="H21" s="63"/>
       <c r="I21" s="13"/>
       <c r="J21" s="13"/>
       <c r="K21" s="13"/>
-      <c r="L21" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="M21" s="60"/>
-      <c r="N21" s="60"/>
-      <c r="O21" s="60"/>
-      <c r="P21" s="60"/>
-      <c r="Q21" s="60"/>
-      <c r="R21" s="60"/>
-      <c r="S21" s="60"/>
-      <c r="T21" s="60"/>
-      <c r="U21" s="60"/>
+      <c r="L21" s="63" t="s">
+        <v>31</v>
+      </c>
+      <c r="M21" s="63"/>
+      <c r="N21" s="63"/>
+      <c r="O21" s="63"/>
+      <c r="P21" s="63"/>
+      <c r="Q21" s="63"/>
+      <c r="R21" s="63"/>
+      <c r="S21" s="63"/>
+      <c r="T21" s="63"/>
+      <c r="U21" s="63"/>
     </row>
     <row r="22" spans="1:21">
-      <c r="A22" s="61" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="61"/>
-      <c r="C22" s="61"/>
-      <c r="D22" s="61"/>
-      <c r="E22" s="61"/>
-      <c r="F22" s="61"/>
-      <c r="G22" s="61"/>
-      <c r="H22" s="61"/>
+      <c r="A22" s="64" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="64"/>
+      <c r="C22" s="64"/>
+      <c r="D22" s="64"/>
+      <c r="E22" s="64"/>
+      <c r="F22" s="64"/>
+      <c r="G22" s="64"/>
+      <c r="H22" s="64"/>
       <c r="I22" s="14"/>
       <c r="J22" s="14"/>
       <c r="K22" s="14"/>
-      <c r="L22" s="51" t="s">
-        <v>22</v>
-      </c>
-      <c r="M22" s="51"/>
-      <c r="N22" s="51"/>
-      <c r="O22" s="51"/>
-      <c r="P22" s="51"/>
-      <c r="Q22" s="51"/>
-      <c r="R22" s="51"/>
-      <c r="S22" s="51"/>
-      <c r="T22" s="51"/>
-      <c r="U22" s="51"/>
+      <c r="L22" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="M22" s="52"/>
+      <c r="N22" s="52"/>
+      <c r="O22" s="52"/>
+      <c r="P22" s="52"/>
+      <c r="Q22" s="52"/>
+      <c r="R22" s="52"/>
+      <c r="S22" s="52"/>
+      <c r="T22" s="52"/>
+      <c r="U22" s="52"/>
     </row>
     <row r="23" spans="1:21" ht="3" customHeight="1">
       <c r="A23" s="2"/>
@@ -1595,7 +1585,7 @@
     </row>
     <row r="24" spans="1:21">
       <c r="A24" s="15" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -1620,7 +1610,7 @@
     </row>
     <row r="25" spans="1:21">
       <c r="A25" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -1633,7 +1623,7 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
@@ -1669,12 +1659,12 @@
       <c r="U26" s="2"/>
     </row>
     <row r="27" spans="1:21">
-      <c r="A27" s="65"/>
-      <c r="B27" s="65"/>
-      <c r="C27" s="65"/>
-      <c r="D27" s="65"/>
-      <c r="E27" s="65"/>
-      <c r="F27" s="65"/>
+      <c r="A27" s="69"/>
+      <c r="B27" s="69"/>
+      <c r="C27" s="69"/>
+      <c r="D27" s="69"/>
+      <c r="E27" s="69"/>
+      <c r="F27" s="69"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
@@ -1692,31 +1682,31 @@
       <c r="U27" s="25"/>
     </row>
     <row r="28" spans="1:21">
-      <c r="A28" s="66" t="s">
-        <v>26</v>
-      </c>
-      <c r="B28" s="66"/>
-      <c r="C28" s="66"/>
-      <c r="D28" s="66"/>
-      <c r="E28" s="66"/>
-      <c r="F28" s="66"/>
+      <c r="A28" s="70" t="s">
+        <v>24</v>
+      </c>
+      <c r="B28" s="70"/>
+      <c r="C28" s="70"/>
+      <c r="D28" s="70"/>
+      <c r="E28" s="70"/>
+      <c r="F28" s="70"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
-      <c r="L28" s="51" t="s">
-        <v>27</v>
-      </c>
-      <c r="M28" s="51"/>
-      <c r="N28" s="51"/>
-      <c r="O28" s="51"/>
-      <c r="P28" s="51"/>
-      <c r="Q28" s="51"/>
-      <c r="R28" s="51"/>
-      <c r="S28" s="51"/>
-      <c r="T28" s="51"/>
-      <c r="U28" s="51"/>
+      <c r="L28" s="52" t="s">
+        <v>25</v>
+      </c>
+      <c r="M28" s="52"/>
+      <c r="N28" s="52"/>
+      <c r="O28" s="52"/>
+      <c r="P28" s="52"/>
+      <c r="Q28" s="52"/>
+      <c r="R28" s="52"/>
+      <c r="S28" s="52"/>
+      <c r="T28" s="52"/>
+      <c r="U28" s="52"/>
     </row>
     <row r="29" spans="1:21">
       <c r="A29" s="16"/>
@@ -1742,37 +1732,37 @@
       <c r="U29" s="16"/>
     </row>
     <row r="31" spans="1:21" ht="20.399999999999999">
-      <c r="A31" s="67"/>
-      <c r="B31" s="67"/>
-      <c r="C31" s="67"/>
-      <c r="D31" s="67"/>
-      <c r="E31" s="67"/>
-      <c r="F31" s="67"/>
-      <c r="G31" s="67"/>
-      <c r="H31" s="67"/>
-      <c r="I31" s="67"/>
-      <c r="J31" s="67"/>
-      <c r="K31" s="67"/>
-      <c r="L31" s="67"/>
-      <c r="M31" s="67"/>
-      <c r="N31" s="67"/>
-      <c r="O31" s="67"/>
-      <c r="P31" s="67"/>
-      <c r="Q31" s="67"/>
-      <c r="R31" s="67"/>
-      <c r="S31" s="67"/>
-      <c r="T31" s="67"/>
-      <c r="U31" s="67"/>
+      <c r="A31" s="71"/>
+      <c r="B31" s="71"/>
+      <c r="C31" s="71"/>
+      <c r="D31" s="71"/>
+      <c r="E31" s="71"/>
+      <c r="F31" s="71"/>
+      <c r="G31" s="71"/>
+      <c r="H31" s="71"/>
+      <c r="I31" s="71"/>
+      <c r="J31" s="71"/>
+      <c r="K31" s="71"/>
+      <c r="L31" s="71"/>
+      <c r="M31" s="71"/>
+      <c r="N31" s="71"/>
+      <c r="O31" s="71"/>
+      <c r="P31" s="71"/>
+      <c r="Q31" s="71"/>
+      <c r="R31" s="71"/>
+      <c r="S31" s="71"/>
+      <c r="T31" s="71"/>
+      <c r="U31" s="71"/>
     </row>
     <row r="33" spans="2:21">
       <c r="N33" s="19"/>
       <c r="S33" s="27"/>
     </row>
     <row r="34" spans="2:21">
-      <c r="H34" s="68"/>
-      <c r="I34" s="68"/>
-      <c r="J34" s="68"/>
-      <c r="K34" s="68"/>
+      <c r="H34" s="72"/>
+      <c r="I34" s="72"/>
+      <c r="J34" s="72"/>
+      <c r="K34" s="72"/>
     </row>
     <row r="35" spans="2:21" ht="15">
       <c r="B35" s="17"/>
@@ -1781,11 +1771,11 @@
     <row r="37" spans="2:21" ht="15">
       <c r="C37" s="19"/>
       <c r="F37" s="19"/>
-      <c r="Q37" s="69"/>
-      <c r="R37" s="69"/>
-      <c r="S37" s="69"/>
-      <c r="T37" s="69"/>
-      <c r="U37" s="69"/>
+      <c r="Q37" s="73"/>
+      <c r="R37" s="73"/>
+      <c r="S37" s="73"/>
+      <c r="T37" s="73"/>
+      <c r="U37" s="73"/>
     </row>
     <row r="39" spans="2:21">
       <c r="C39" s="19"/>
@@ -1799,92 +1789,92 @@
     </row>
     <row r="44" spans="2:21">
       <c r="E44" s="21"/>
-      <c r="H44" s="70"/>
-      <c r="I44" s="70"/>
+      <c r="H44" s="74"/>
+      <c r="I44" s="74"/>
     </row>
     <row r="45" spans="2:21">
       <c r="E45" s="21"/>
-      <c r="H45" s="70"/>
-      <c r="I45" s="70"/>
+      <c r="H45" s="74"/>
+      <c r="I45" s="74"/>
     </row>
     <row r="46" spans="2:21">
       <c r="E46" s="22"/>
-      <c r="H46" s="70"/>
-      <c r="I46" s="70"/>
+      <c r="H46" s="74"/>
+      <c r="I46" s="74"/>
       <c r="R46" s="17"/>
       <c r="S46" s="17"/>
       <c r="T46" s="17"/>
       <c r="U46" s="17"/>
     </row>
     <row r="47" spans="2:21">
-      <c r="H47" s="70"/>
-      <c r="I47" s="70"/>
+      <c r="H47" s="74"/>
+      <c r="I47" s="74"/>
       <c r="R47" s="17"/>
       <c r="S47" s="17"/>
       <c r="T47" s="17"/>
       <c r="U47" s="17"/>
     </row>
     <row r="48" spans="2:21">
-      <c r="H48" s="71"/>
-      <c r="I48" s="71"/>
+      <c r="H48" s="75"/>
+      <c r="I48" s="75"/>
     </row>
     <row r="52" spans="1:21">
-      <c r="A52" s="64"/>
-      <c r="B52" s="64"/>
-      <c r="C52" s="64"/>
-      <c r="D52" s="64"/>
-      <c r="E52" s="64"/>
-      <c r="F52" s="64"/>
+      <c r="A52" s="68"/>
+      <c r="B52" s="68"/>
+      <c r="C52" s="68"/>
+      <c r="D52" s="68"/>
+      <c r="E52" s="68"/>
+      <c r="F52" s="68"/>
     </row>
     <row r="53" spans="1:21">
-      <c r="A53" s="64"/>
-      <c r="B53" s="64"/>
-      <c r="C53" s="64"/>
-      <c r="D53" s="64"/>
-      <c r="E53" s="64"/>
-      <c r="F53" s="64"/>
-      <c r="L53" s="64"/>
-      <c r="M53" s="64"/>
-      <c r="N53" s="64"/>
-      <c r="O53" s="64"/>
-      <c r="P53" s="64"/>
-      <c r="Q53" s="64"/>
-      <c r="R53" s="64"/>
-      <c r="S53" s="64"/>
-      <c r="T53" s="64"/>
-      <c r="U53" s="64"/>
+      <c r="A53" s="68"/>
+      <c r="B53" s="68"/>
+      <c r="C53" s="68"/>
+      <c r="D53" s="68"/>
+      <c r="E53" s="68"/>
+      <c r="F53" s="68"/>
+      <c r="L53" s="68"/>
+      <c r="M53" s="68"/>
+      <c r="N53" s="68"/>
+      <c r="O53" s="68"/>
+      <c r="P53" s="68"/>
+      <c r="Q53" s="68"/>
+      <c r="R53" s="68"/>
+      <c r="S53" s="68"/>
+      <c r="T53" s="68"/>
+      <c r="U53" s="68"/>
     </row>
     <row r="55" spans="1:21">
       <c r="A55" s="23"/>
     </row>
     <row r="58" spans="1:21">
-      <c r="A58" s="64"/>
-      <c r="B58" s="64"/>
-      <c r="C58" s="64"/>
-      <c r="D58" s="64"/>
-      <c r="E58" s="64"/>
-      <c r="F58" s="64"/>
+      <c r="A58" s="68"/>
+      <c r="B58" s="68"/>
+      <c r="C58" s="68"/>
+      <c r="D58" s="68"/>
+      <c r="E58" s="68"/>
+      <c r="F58" s="68"/>
     </row>
     <row r="59" spans="1:21">
-      <c r="A59" s="64"/>
-      <c r="B59" s="64"/>
-      <c r="C59" s="64"/>
-      <c r="D59" s="64"/>
-      <c r="E59" s="64"/>
-      <c r="F59" s="64"/>
-      <c r="L59" s="64"/>
-      <c r="M59" s="64"/>
-      <c r="N59" s="64"/>
-      <c r="O59" s="64"/>
-      <c r="P59" s="64"/>
-      <c r="Q59" s="64"/>
-      <c r="R59" s="64"/>
-      <c r="S59" s="64"/>
-      <c r="T59" s="64"/>
-      <c r="U59" s="64"/>
+      <c r="A59" s="68"/>
+      <c r="B59" s="68"/>
+      <c r="C59" s="68"/>
+      <c r="D59" s="68"/>
+      <c r="E59" s="68"/>
+      <c r="F59" s="68"/>
+      <c r="L59" s="68"/>
+      <c r="M59" s="68"/>
+      <c r="N59" s="68"/>
+      <c r="O59" s="68"/>
+      <c r="P59" s="68"/>
+      <c r="Q59" s="68"/>
+      <c r="R59" s="68"/>
+      <c r="S59" s="68"/>
+      <c r="T59" s="68"/>
+      <c r="U59" s="68"/>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="31">
     <mergeCell ref="A53:F53"/>
     <mergeCell ref="L53:U53"/>
     <mergeCell ref="A58:F58"/>
@@ -1915,6 +1905,7 @@
     <mergeCell ref="N17:S17"/>
     <mergeCell ref="H18:I18"/>
     <mergeCell ref="L21:U21"/>
+    <mergeCell ref="T15:U15"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.196850393700787" right="0.196850393700787" top="0.39370078740157499" bottom="0.196850393700787" header="0.31496062992126" footer="0.31496062992126"/>

</xml_diff>